<commit_message>
WHatsapp, sms and export validator files working
</commit_message>
<xml_diff>
--- a/Duplicate_Transactions.xlsx
+++ b/Duplicate_Transactions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N432"/>
+  <dimension ref="A1:N475"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22023,10 +22023,8 @@
           <t>Dennis Vanmeter</t>
         </is>
       </c>
-      <c r="B432" t="inlineStr">
-        <is>
-          <t>13049196111</t>
-        </is>
+      <c r="B432" t="n">
+        <v>13049196111</v>
       </c>
       <c r="C432" t="inlineStr">
         <is>
@@ -22069,6 +22067,2158 @@
         </is>
       </c>
     </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Madhukar Verma</t>
+        </is>
+      </c>
+      <c r="B433" t="n">
+        <v>2065044242</v>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>42729 Mayfair Park Ave Fremont Fremont 94538 California USA</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr"/>
+      <c r="G433" t="inlineStr"/>
+      <c r="H433" t="inlineStr"/>
+      <c r="I433" t="inlineStr"/>
+      <c r="J433" t="inlineStr"/>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:09:43</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N433" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B434" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr"/>
+      <c r="G434" t="inlineStr"/>
+      <c r="H434" t="inlineStr"/>
+      <c r="I434" t="inlineStr"/>
+      <c r="J434" t="inlineStr"/>
+      <c r="K434" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:09:46</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N434" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B435" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr"/>
+      <c r="G435" t="inlineStr"/>
+      <c r="H435" t="inlineStr"/>
+      <c r="I435" t="inlineStr"/>
+      <c r="J435" t="inlineStr"/>
+      <c r="K435" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:09:49</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N435" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B436" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr"/>
+      <c r="G436" t="inlineStr"/>
+      <c r="H436" t="inlineStr"/>
+      <c r="I436" t="inlineStr"/>
+      <c r="J436" t="inlineStr"/>
+      <c r="K436" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:09:51</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N436" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Madhukar Verma</t>
+        </is>
+      </c>
+      <c r="B437" t="n">
+        <v>2065044242</v>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>42729 Mayfair Park Ave Fremont Fremont 94538 California USA</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr"/>
+      <c r="G437" t="inlineStr"/>
+      <c r="H437" t="inlineStr"/>
+      <c r="I437" t="inlineStr"/>
+      <c r="J437" t="inlineStr"/>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:15:09</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N437" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B438" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr"/>
+      <c r="G438" t="inlineStr"/>
+      <c r="H438" t="inlineStr"/>
+      <c r="I438" t="inlineStr"/>
+      <c r="J438" t="inlineStr"/>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:15:12</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N438" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B439" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr"/>
+      <c r="G439" t="inlineStr"/>
+      <c r="H439" t="inlineStr"/>
+      <c r="I439" t="inlineStr"/>
+      <c r="J439" t="inlineStr"/>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:15:15</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N439" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B440" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr"/>
+      <c r="G440" t="inlineStr"/>
+      <c r="H440" t="inlineStr"/>
+      <c r="I440" t="inlineStr"/>
+      <c r="J440" t="inlineStr"/>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:15:17</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N440" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B441" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr"/>
+      <c r="G441" t="inlineStr"/>
+      <c r="H441" t="inlineStr"/>
+      <c r="I441" t="inlineStr"/>
+      <c r="J441" t="inlineStr"/>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:16:17</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N441" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B442" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr"/>
+      <c r="G442" t="inlineStr"/>
+      <c r="H442" t="inlineStr"/>
+      <c r="I442" t="inlineStr"/>
+      <c r="J442" t="inlineStr"/>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:16:20</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N442" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B443" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr"/>
+      <c r="G443" t="inlineStr"/>
+      <c r="H443" t="inlineStr"/>
+      <c r="I443" t="inlineStr"/>
+      <c r="J443" t="inlineStr"/>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:16:23</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N443" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Madhukar Verma</t>
+        </is>
+      </c>
+      <c r="B444" t="n">
+        <v>2065044242</v>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>42729 Mayfair Park Ave Fremont Fremont 94538 California USA</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>BSBT</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr"/>
+      <c r="G444" t="inlineStr"/>
+      <c r="H444" t="inlineStr"/>
+      <c r="I444" t="inlineStr"/>
+      <c r="J444" t="inlineStr"/>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:16:47</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N444" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B445" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr"/>
+      <c r="G445" t="inlineStr"/>
+      <c r="H445" t="inlineStr"/>
+      <c r="I445" t="inlineStr"/>
+      <c r="J445" t="inlineStr"/>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:16:50</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N445" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B446" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr"/>
+      <c r="G446" t="inlineStr"/>
+      <c r="H446" t="inlineStr"/>
+      <c r="I446" t="inlineStr"/>
+      <c r="J446" t="inlineStr"/>
+      <c r="K446" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:16:53</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N446" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B447" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr"/>
+      <c r="G447" t="inlineStr"/>
+      <c r="H447" t="inlineStr"/>
+      <c r="I447" t="inlineStr"/>
+      <c r="J447" t="inlineStr"/>
+      <c r="K447" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:16:56</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N447" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B448" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr"/>
+      <c r="G448" t="inlineStr"/>
+      <c r="H448" t="inlineStr"/>
+      <c r="I448" t="inlineStr"/>
+      <c r="J448" t="inlineStr"/>
+      <c r="K448" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:18:21</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N448" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B449" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr"/>
+      <c r="G449" t="inlineStr"/>
+      <c r="H449" t="inlineStr"/>
+      <c r="I449" t="inlineStr"/>
+      <c r="J449" t="inlineStr"/>
+      <c r="K449" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:18:23</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N449" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B450" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr"/>
+      <c r="G450" t="inlineStr"/>
+      <c r="H450" t="inlineStr"/>
+      <c r="I450" t="inlineStr"/>
+      <c r="J450" t="inlineStr"/>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:18:25</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N450" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B451" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr"/>
+      <c r="G451" t="inlineStr"/>
+      <c r="H451" t="inlineStr"/>
+      <c r="I451" t="inlineStr"/>
+      <c r="J451" t="inlineStr"/>
+      <c r="K451" t="inlineStr">
+        <is>
+          <t>Both SMS and WhatsApp messages already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:23:45</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N451" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B452" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr"/>
+      <c r="G452" t="inlineStr"/>
+      <c r="H452" t="inlineStr"/>
+      <c r="I452" t="inlineStr"/>
+      <c r="J452" t="inlineStr"/>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t>Both SMS and WhatsApp messages already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:23:48</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N452" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B453" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr"/>
+      <c r="G453" t="inlineStr"/>
+      <c r="H453" t="inlineStr"/>
+      <c r="I453" t="inlineStr"/>
+      <c r="J453" t="inlineStr"/>
+      <c r="K453" t="inlineStr">
+        <is>
+          <t>Both SMS and WhatsApp messages already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:23:51</t>
+        </is>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N453" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B454" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr"/>
+      <c r="G454" t="inlineStr"/>
+      <c r="H454" t="inlineStr"/>
+      <c r="I454" t="inlineStr"/>
+      <c r="J454" t="inlineStr"/>
+      <c r="K454" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:24:34</t>
+        </is>
+      </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N454" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B455" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr"/>
+      <c r="G455" t="inlineStr"/>
+      <c r="H455" t="inlineStr"/>
+      <c r="I455" t="inlineStr"/>
+      <c r="J455" t="inlineStr"/>
+      <c r="K455" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:24:36</t>
+        </is>
+      </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N455" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B456" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr"/>
+      <c r="G456" t="inlineStr"/>
+      <c r="H456" t="inlineStr"/>
+      <c r="I456" t="inlineStr"/>
+      <c r="J456" t="inlineStr"/>
+      <c r="K456" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:24:38</t>
+        </is>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N456" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Madhukar Verma</t>
+        </is>
+      </c>
+      <c r="B457" t="n">
+        <v>2065044242</v>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>42729 Mayfair Park Ave Fremont Fremont 94538 California USA</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>BSBT</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr"/>
+      <c r="G457" t="inlineStr"/>
+      <c r="H457" t="inlineStr"/>
+      <c r="I457" t="inlineStr"/>
+      <c r="J457" t="inlineStr"/>
+      <c r="K457" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:30:51</t>
+        </is>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N457" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B458" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr"/>
+      <c r="G458" t="inlineStr"/>
+      <c r="H458" t="inlineStr"/>
+      <c r="I458" t="inlineStr"/>
+      <c r="J458" t="inlineStr"/>
+      <c r="K458" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:30:54</t>
+        </is>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N458" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B459" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr"/>
+      <c r="G459" t="inlineStr"/>
+      <c r="H459" t="inlineStr"/>
+      <c r="I459" t="inlineStr"/>
+      <c r="J459" t="inlineStr"/>
+      <c r="K459" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:30:57</t>
+        </is>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N459" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B460" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr"/>
+      <c r="G460" t="inlineStr"/>
+      <c r="H460" t="inlineStr"/>
+      <c r="I460" t="inlineStr"/>
+      <c r="J460" t="inlineStr"/>
+      <c r="K460" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:31:00</t>
+        </is>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N460" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B461" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr"/>
+      <c r="G461" t="inlineStr"/>
+      <c r="H461" t="inlineStr"/>
+      <c r="I461" t="inlineStr"/>
+      <c r="J461" t="inlineStr"/>
+      <c r="K461" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:32:15</t>
+        </is>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N461" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B462" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr"/>
+      <c r="G462" t="inlineStr"/>
+      <c r="H462" t="inlineStr"/>
+      <c r="I462" t="inlineStr"/>
+      <c r="J462" t="inlineStr"/>
+      <c r="K462" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:32:18</t>
+        </is>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N462" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B463" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr"/>
+      <c r="G463" t="inlineStr"/>
+      <c r="H463" t="inlineStr"/>
+      <c r="I463" t="inlineStr"/>
+      <c r="J463" t="inlineStr"/>
+      <c r="K463" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:32:21</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N463" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>Madhukar Verma</t>
+        </is>
+      </c>
+      <c r="B464" t="n">
+        <v>2065044242</v>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>42729 Mayfair Park Ave Fremont Fremont 94538 California USA</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>JKR</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr"/>
+      <c r="G464" t="inlineStr"/>
+      <c r="H464" t="inlineStr"/>
+      <c r="I464" t="inlineStr"/>
+      <c r="J464" t="inlineStr"/>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:33:32</t>
+        </is>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N464" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B465" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr"/>
+      <c r="G465" t="inlineStr"/>
+      <c r="H465" t="inlineStr"/>
+      <c r="I465" t="inlineStr"/>
+      <c r="J465" t="inlineStr"/>
+      <c r="K465" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:33:34</t>
+        </is>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N465" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B466" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr"/>
+      <c r="G466" t="inlineStr"/>
+      <c r="H466" t="inlineStr"/>
+      <c r="I466" t="inlineStr"/>
+      <c r="J466" t="inlineStr"/>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:33:37</t>
+        </is>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N466" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B467" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr"/>
+      <c r="G467" t="inlineStr"/>
+      <c r="H467" t="inlineStr"/>
+      <c r="I467" t="inlineStr"/>
+      <c r="J467" t="inlineStr"/>
+      <c r="K467" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:33:40</t>
+        </is>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N467" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Madhukar Verma</t>
+        </is>
+      </c>
+      <c r="B468" t="n">
+        <v>2065044242</v>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>42729 Mayfair Park Ave Fremont Fremont 94538 California USA</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>JKR</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr"/>
+      <c r="G468" t="inlineStr"/>
+      <c r="H468" t="inlineStr"/>
+      <c r="I468" t="inlineStr"/>
+      <c r="J468" t="inlineStr"/>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:35:19</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N468" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B469" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr"/>
+      <c r="G469" t="inlineStr"/>
+      <c r="H469" t="inlineStr"/>
+      <c r="I469" t="inlineStr"/>
+      <c r="J469" t="inlineStr"/>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:35:21</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N469" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B470" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr"/>
+      <c r="G470" t="inlineStr"/>
+      <c r="H470" t="inlineStr"/>
+      <c r="I470" t="inlineStr"/>
+      <c r="J470" t="inlineStr"/>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:35:24</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N470" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B471" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr"/>
+      <c r="G471" t="inlineStr"/>
+      <c r="H471" t="inlineStr"/>
+      <c r="I471" t="inlineStr"/>
+      <c r="J471" t="inlineStr"/>
+      <c r="K471" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:35:27</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N471" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Madhukar Verma</t>
+        </is>
+      </c>
+      <c r="B472" t="n">
+        <v>2065044242</v>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>42729 Mayfair Park Ave Fremont Fremont 94538 California USA</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>JKR</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr"/>
+      <c r="G472" t="inlineStr"/>
+      <c r="H472" t="inlineStr"/>
+      <c r="I472" t="inlineStr"/>
+      <c r="J472" t="inlineStr"/>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:35:45</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N472" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B473" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr"/>
+      <c r="G473" t="inlineStr"/>
+      <c r="H473" t="inlineStr"/>
+      <c r="I473" t="inlineStr"/>
+      <c r="J473" t="inlineStr"/>
+      <c r="K473" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:35:48</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N473" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B474" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr"/>
+      <c r="G474" t="inlineStr"/>
+      <c r="H474" t="inlineStr"/>
+      <c r="I474" t="inlineStr"/>
+      <c r="J474" t="inlineStr"/>
+      <c r="K474" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:35:51</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N474" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>13049196111</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr"/>
+      <c r="G475" t="inlineStr"/>
+      <c r="H475" t="inlineStr"/>
+      <c r="I475" t="inlineStr"/>
+      <c r="J475" t="inlineStr"/>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>2025-09-20 14:35:54</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N475" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
IMplemented voip block using twillio apis
</commit_message>
<xml_diff>
--- a/Duplicate_Transactions.xlsx
+++ b/Duplicate_Transactions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N475"/>
+  <dimension ref="A1:N483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24173,10 +24173,8 @@
           <t>Dennis Vanmeter</t>
         </is>
       </c>
-      <c r="B475" t="inlineStr">
-        <is>
-          <t>13049196111</t>
-        </is>
+      <c r="B475" t="n">
+        <v>13049196111</v>
       </c>
       <c r="C475" t="inlineStr">
         <is>
@@ -24219,6 +24217,408 @@
         </is>
       </c>
     </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Madhukar Verma</t>
+        </is>
+      </c>
+      <c r="B476" t="n">
+        <v>2065044242</v>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>42729 Mayfair Park Ave Fremont Fremont 94538 California USA</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>JKR</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr"/>
+      <c r="G476" t="inlineStr"/>
+      <c r="H476" t="inlineStr"/>
+      <c r="I476" t="inlineStr"/>
+      <c r="J476" t="inlineStr"/>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>2025-09-20 15:02:05</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N476" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B477" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr"/>
+      <c r="G477" t="inlineStr"/>
+      <c r="H477" t="inlineStr"/>
+      <c r="I477" t="inlineStr"/>
+      <c r="J477" t="inlineStr"/>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>2025-09-20 15:02:08</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N477" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B478" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr"/>
+      <c r="G478" t="inlineStr"/>
+      <c r="H478" t="inlineStr"/>
+      <c r="I478" t="inlineStr"/>
+      <c r="J478" t="inlineStr"/>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>2025-09-20 15:02:10</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N478" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B479" t="n">
+        <v>13049196111</v>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr"/>
+      <c r="G479" t="inlineStr"/>
+      <c r="H479" t="inlineStr"/>
+      <c r="I479" t="inlineStr"/>
+      <c r="J479" t="inlineStr"/>
+      <c r="K479" t="inlineStr">
+        <is>
+          <t>WhatsApp message already sent for this book previously</t>
+        </is>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>2025-09-20 15:02:13</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N479" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Madhukar Verma</t>
+        </is>
+      </c>
+      <c r="B480" t="n">
+        <v>2065044242</v>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>42729 Mayfair Park Ave Fremont Fremont 94538 California USA</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>JKR</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr"/>
+      <c r="G480" t="inlineStr"/>
+      <c r="H480" t="inlineStr"/>
+      <c r="I480" t="inlineStr"/>
+      <c r="J480" t="inlineStr"/>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>2025-09-20 15:02:32</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N480" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B481" t="n">
+        <v>12814104622</v>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>PO Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Po Box 87301, Park Place, Houston, Texas</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr"/>
+      <c r="G481" t="inlineStr"/>
+      <c r="H481" t="inlineStr"/>
+      <c r="I481" t="inlineStr"/>
+      <c r="J481" t="inlineStr"/>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>2025-09-20 15:02:35</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N481" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Henry Chelegbor</t>
+        </is>
+      </c>
+      <c r="B482" t="n">
+        <v>13024705411</v>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, PA, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>6613 Guyer Street, Philadelphia, Pa, Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr"/>
+      <c r="G482" t="inlineStr"/>
+      <c r="H482" t="inlineStr"/>
+      <c r="I482" t="inlineStr"/>
+      <c r="J482" t="inlineStr"/>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>2025-09-20 15:02:38</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N482" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Dennis Vanmeter</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>13049196111</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, WV 25801</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>1909 Harper Rd, Beckley, Wv 25801</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr"/>
+      <c r="G483" t="inlineStr"/>
+      <c r="H483" t="inlineStr"/>
+      <c r="I483" t="inlineStr"/>
+      <c r="J483" t="inlineStr"/>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>Same book already sent</t>
+        </is>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>2025-09-20 15:02:40</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>2025-09-20</t>
+        </is>
+      </c>
+      <c r="N483" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>